<commit_message>
Refactor category covers to category.xlsx + category modal updates
- Move word & phrase category covers out of WordList.xlsx into category.xlsx
  (2 sheets: Categories + Phrase Categories)
- sync-data.mjs: reads/writes covers+order from category.xlsx exclusively;
  WordList.xlsx Covers/Phrase Covers sheets removed
- Category modal: hide Level tab, rename Theme→Words, add All card
- Data sync: 248 words · 198 phrases

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/update_data_folder/category.xlsx
+++ b/update_data_folder/category.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miaofang/Desktop/VocabWorkspace/update_data_folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B05235A-570B-DA4F-BB73-C411C14FEF56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B18925-ADB2-C94E-A802-801F675098D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Categories" sheetId="1" r:id="rId1"/>
+    <sheet name="Phrase Categories" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Categories!$A$1:$F$14</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>Category</t>
   </si>
@@ -49,12 +50,18 @@
     <t>Verb</t>
   </si>
   <si>
+    <t>eat</t>
+  </si>
+  <si>
     <t>Adjective</t>
   </si>
   <si>
     <t>Emotion, Quality, Sensation, Size</t>
   </si>
   <si>
+    <t>cheap</t>
+  </si>
+  <si>
     <t>Animal</t>
   </si>
   <si>
@@ -67,6 +74,9 @@
     <t>Color</t>
   </si>
   <si>
+    <t>pink</t>
+  </si>
+  <si>
     <t>Day</t>
   </si>
   <si>
@@ -91,6 +101,9 @@
     <t>Landscape, Plant, Weather&amp;Sky</t>
   </si>
   <si>
+    <t>wind</t>
+  </si>
+  <si>
     <t>Number</t>
   </si>
   <si>
@@ -103,46 +116,55 @@
     <t>Fun, Furniture, Kitchen, Misc, Tech, Tool</t>
   </si>
   <si>
+    <t>trophy</t>
+  </si>
+  <si>
     <t>People</t>
   </si>
   <si>
     <t>Body, Clothing, Family, Job</t>
   </si>
   <si>
+    <t>sister</t>
+  </si>
+  <si>
     <t>Place</t>
   </si>
   <si>
     <t>City, Country, Home, Landmark, Place, Structure</t>
   </si>
   <si>
+    <t>bank</t>
+  </si>
+  <si>
+    <t>today</t>
+  </si>
+  <si>
     <t>Transport</t>
   </si>
   <si>
-    <t>wind</t>
-  </si>
-  <si>
-    <t>cheap</t>
-  </si>
-  <si>
-    <t>today</t>
-  </si>
-  <si>
-    <t>sister</t>
-  </si>
-  <si>
     <t>taxi</t>
   </si>
   <si>
-    <t>bank</t>
-  </si>
-  <si>
-    <t>trophy</t>
-  </si>
-  <si>
-    <t>pink</t>
-  </si>
-  <si>
-    <t>eat</t>
+    <t>everyday</t>
+  </si>
+  <si>
+    <t>orange</t>
+  </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>opinions</t>
+  </si>
+  <si>
+    <t>emotions</t>
+  </si>
+  <si>
+    <t>durian</t>
+  </si>
+  <si>
+    <t>pineapple</t>
   </si>
 </sst>
 </file>
@@ -536,7 +558,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2">
         <v>49</v>
@@ -550,13 +572,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2">
         <v>59</v>
@@ -570,13 +592,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2">
         <v>38</v>
@@ -590,13 +612,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D5" s="2">
         <v>10</v>
@@ -610,13 +632,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D6" s="2">
         <v>7</v>
@@ -630,13 +652,13 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D7" s="2">
         <v>69</v>
@@ -650,13 +672,13 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D8" s="2">
         <v>31</v>
@@ -670,13 +692,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D9" s="2">
         <v>11</v>
@@ -690,13 +712,13 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D10" s="2">
         <v>75</v>
@@ -710,13 +732,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D11" s="2">
         <v>56</v>
@@ -730,10 +752,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
         <v>36</v>
@@ -750,13 +772,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D13" s="2">
         <v>18</v>
@@ -770,13 +792,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D14" s="2">
         <v>18</v>
@@ -792,4 +814,58 @@
   <autoFilter ref="A1:F14" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>